<commit_message>
feat: update Calculo de Consumo por CDN.xlsx with new data
</commit_message>
<xml_diff>
--- a/documents/Calculo de Consumo por CDN.xlsx
+++ b/documents/Calculo de Consumo por CDN.xlsx
@@ -5,15 +5,15 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario pc\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\Laravel\SCOTT\documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F374A41-AC14-46B0-8FBF-48790A863B46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8302B3CB-C959-4C83-B55C-C60CB15A3E63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="BPK Abril 2026" sheetId="1" r:id="rId1"/>
+    <sheet name="BPK" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t>Descripción</t>
   </si>
@@ -83,7 +83,10 @@
     <t>Costo por Dispositivo</t>
   </si>
   <si>
-    <t>Costo Por Usuario</t>
+    <t>Costo por Usuario</t>
+  </si>
+  <si>
+    <t>Costo por Usuarios Totales</t>
   </si>
 </sst>
 </file>
@@ -168,7 +171,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -217,11 +220,61 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -239,13 +292,22 @@
     <xf numFmtId="3" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="4" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="166" fontId="1" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -255,16 +317,16 @@
     <xf numFmtId="166" fontId="4" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="3" fontId="4" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="4" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="4" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -485,10 +547,10 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="59" customWidth="1"/>
+    <col min="1" max="1" width="61.33203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14.109375" customWidth="1"/>
     <col min="3" max="3" width="17.21875" customWidth="1"/>
   </cols>
@@ -509,10 +571,10 @@
         <v>3</v>
       </c>
       <c r="B2" s="5">
-        <v>3420</v>
+        <v>3772</v>
       </c>
       <c r="C2" s="5">
-        <v>7224</v>
+        <v>8109</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -532,136 +594,148 @@
       </c>
       <c r="B4" s="8">
         <f t="shared" ref="B4:C4" si="0">B2*B3</f>
-        <v>10260</v>
+        <v>11316</v>
       </c>
       <c r="C4" s="8">
         <f t="shared" si="0"/>
-        <v>14448</v>
+        <v>16218</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="15">
+      <c r="B5" s="9">
         <f>B2+C2</f>
-        <v>10644</v>
-      </c>
-      <c r="C5" s="11"/>
+        <v>11881</v>
+      </c>
+      <c r="C5" s="10"/>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="15">
+      <c r="B6" s="9">
         <f>B4+C4</f>
-        <v>24708</v>
-      </c>
-      <c r="C6" s="11"/>
+        <v>27534</v>
+      </c>
+      <c r="C6" s="10"/>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="16">
+      <c r="B7" s="11">
         <v>3</v>
       </c>
-      <c r="C7" s="11"/>
+      <c r="C7" s="10"/>
     </row>
     <row r="8" spans="1:3">
       <c r="A8" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="17">
+      <c r="B8" s="12">
         <f>B7*60*60/8/1024</f>
         <v>1.318359375</v>
       </c>
-      <c r="C8" s="11"/>
+      <c r="C8" s="10"/>
     </row>
     <row r="9" spans="1:3">
       <c r="A9" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="18">
+      <c r="B9" s="13">
         <f>(B11/B6)*(1024)</f>
-        <v>21.474919917927039</v>
-      </c>
-      <c r="C9" s="11"/>
+        <v>32.117607579863353</v>
+      </c>
+      <c r="C9" s="10"/>
     </row>
     <row r="10" spans="1:3">
       <c r="A10" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B10" s="12">
-        <v>482580</v>
-      </c>
-      <c r="C10" s="11"/>
+      <c r="B10" s="15">
+        <v>804290</v>
+      </c>
+      <c r="C10" s="10"/>
     </row>
     <row r="11" spans="1:3">
       <c r="A11" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B11" s="13">
+      <c r="B11" s="16">
         <f>B10/931.32257461548</f>
-        <v>518.16632942591923</v>
-      </c>
-      <c r="C11" s="11"/>
+        <v>863.59981162495865</v>
+      </c>
+      <c r="C11" s="10"/>
     </row>
     <row r="12" spans="1:3">
       <c r="A12" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B12" s="10">
+      <c r="B12" s="14">
         <v>75000</v>
       </c>
-      <c r="C12" s="11"/>
+      <c r="C12" s="10"/>
     </row>
     <row r="13" spans="1:3">
       <c r="A13" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B13" s="14">
+      <c r="B13" s="17">
         <f>B12/B11</f>
-        <v>144.74116850296531</v>
-      </c>
-      <c r="C13" s="11"/>
+        <v>86.845780870284344</v>
+      </c>
+      <c r="C13" s="10"/>
     </row>
     <row r="14" spans="1:3">
-      <c r="A14" s="1" t="s">
+      <c r="A14" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="B14" s="14">
+      <c r="B14" s="19">
         <f>B12/B6</f>
-        <v>3.0354541039339487</v>
-      </c>
-      <c r="C14" s="11"/>
+        <v>2.7239049901939421</v>
+      </c>
+      <c r="C14" s="20"/>
     </row>
     <row r="15" spans="1:3">
-      <c r="A15" s="1" t="s">
+      <c r="A15" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="B15" s="9">
+      <c r="B15" s="22">
         <f>B14*B3</f>
-        <v>9.1063623118018455</v>
-      </c>
-      <c r="C15" s="9">
+        <v>8.1717149705818262</v>
+      </c>
+      <c r="C15" s="22">
         <f>B14*C3</f>
-        <v>6.0709082078678973</v>
-      </c>
+        <v>5.4478099803878841</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A16" s="21" t="s">
+        <v>17</v>
+      </c>
+      <c r="B16" s="23">
+        <f>B12/B5</f>
+        <v>6.3125999494992007</v>
+      </c>
+      <c r="C16" s="23"/>
     </row>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="11">
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="B14:C14"/>
     <mergeCell ref="B5:C5"/>
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="B7:C7"/>
     <mergeCell ref="B8:C8"/>
     <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="B14:C14"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: Enhance solar interference modal with progress tracking and search functionality
</commit_message>
<xml_diff>
--- a/documents/Calculo de Consumo por CDN.xlsx
+++ b/documents/Calculo de Consumo por CDN.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\Laravel\SCOTT\documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F74975A6-4D14-4584-AE18-BE67B6FC8AB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EED04426-EC60-415A-BD1D-06DB6384C05E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
   <si>
     <t>Descripción</t>
   </si>
@@ -87,6 +87,15 @@
   </si>
   <si>
     <t>Costo por Usuarios Totales</t>
+  </si>
+  <si>
+    <t>Total de Horas Consumidas al Mes</t>
+  </si>
+  <si>
+    <t>Horas Promedio de Consumo por Dispositivo</t>
+  </si>
+  <si>
+    <t>Horas Promedio de Consumo por Suscriptor</t>
   </si>
 </sst>
 </file>
@@ -274,7 +283,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -297,16 +306,25 @@
     <xf numFmtId="166" fontId="4" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="3" fontId="4" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="166" fontId="4" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="166" fontId="1" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="165" fontId="4" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -317,16 +335,13 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="4" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="1" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="4" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -547,7 +562,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="61.33203125" bestFit="1" customWidth="1"/>
@@ -605,98 +620,98 @@
       <c r="A5" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="20">
+      <c r="B5" s="12">
         <f>B2+C2</f>
         <v>13074</v>
       </c>
-      <c r="C5" s="14"/>
+      <c r="C5" s="13"/>
     </row>
     <row r="6" spans="1:3" ht="13.2">
       <c r="A6" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="20">
+      <c r="B6" s="12">
         <f>B4+C4</f>
         <v>31199</v>
       </c>
-      <c r="C6" s="14"/>
+      <c r="C6" s="13"/>
     </row>
     <row r="7" spans="1:3" ht="13.2">
       <c r="A7" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="21">
+      <c r="B7" s="14">
         <v>3</v>
       </c>
-      <c r="C7" s="14"/>
+      <c r="C7" s="13"/>
     </row>
     <row r="8" spans="1:3" ht="13.2">
       <c r="A8" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="22">
+      <c r="B8" s="15">
         <f>B7*60*60/8/1024</f>
         <v>1.318359375</v>
       </c>
-      <c r="C8" s="14"/>
+      <c r="C8" s="13"/>
     </row>
     <row r="9" spans="1:3" ht="13.2">
       <c r="A9" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="23">
+      <c r="B9" s="16">
         <f>(B11/B6)*(1024)</f>
-        <v>34.772817334219035</v>
-      </c>
-      <c r="C9" s="14"/>
+        <v>35.241886848168157</v>
+      </c>
+      <c r="C9" s="13"/>
     </row>
     <row r="10" spans="1:3" ht="13.2">
       <c r="A10" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B10" s="15">
-        <v>986690</v>
-      </c>
-      <c r="C10" s="14"/>
+      <c r="B10" s="23">
+        <v>1000000</v>
+      </c>
+      <c r="C10" s="13"/>
     </row>
     <row r="11" spans="1:3" ht="13.2">
       <c r="A11" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B11" s="16">
+      <c r="B11" s="19">
         <f>B10/931.32257461548</f>
-        <v>1059.4503203225584</v>
-      </c>
-      <c r="C11" s="14"/>
+        <v>1073.7418239999984</v>
+      </c>
+      <c r="C11" s="13"/>
     </row>
     <row r="12" spans="1:3" ht="13.2">
       <c r="A12" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B12" s="13">
+      <c r="B12" s="18">
         <v>75000</v>
       </c>
-      <c r="C12" s="14"/>
+      <c r="C12" s="13"/>
     </row>
     <row r="13" spans="1:3" ht="13.2">
       <c r="A13" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B13" s="17">
+      <c r="B13" s="20">
         <f>B12/B11</f>
-        <v>70.791426989389777</v>
-      </c>
-      <c r="C13" s="14"/>
+        <v>69.849193096161002</v>
+      </c>
+      <c r="C13" s="13"/>
     </row>
     <row r="14" spans="1:3" ht="13.2">
       <c r="A14" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="B14" s="18">
+      <c r="B14" s="21">
         <f>B12/B6</f>
         <v>2.4039232026667521</v>
       </c>
-      <c r="C14" s="19"/>
+      <c r="C14" s="22"/>
     </row>
     <row r="15" spans="1:3" ht="13.2">
       <c r="A15" s="10" t="s">
@@ -715,25 +730,57 @@
       <c r="A16" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="B16" s="12">
+      <c r="B16" s="17">
         <f>B12/B5</f>
         <v>5.736576411197797</v>
       </c>
-      <c r="C16" s="12"/>
+      <c r="C16" s="17"/>
+    </row>
+    <row r="17" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A17" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="B17" s="25">
+        <v>390076.98</v>
+      </c>
+      <c r="C17" s="25"/>
+    </row>
+    <row r="18" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A18" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="B18" s="24">
+        <f>B17/B6</f>
+        <v>12.502868040642328</v>
+      </c>
+      <c r="C18" s="24"/>
+    </row>
+    <row r="19" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A19" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="B19" s="24">
+        <f>B17/B5</f>
+        <v>29.836085360256998</v>
+      </c>
+      <c r="C19" s="24"/>
     </row>
   </sheetData>
-  <mergeCells count="11">
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="B7:C7"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="B9:C9"/>
+  <mergeCells count="14">
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="B19:C19"/>
     <mergeCell ref="B16:C16"/>
     <mergeCell ref="B12:C12"/>
     <mergeCell ref="B10:C10"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="B9:C9"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
feat: Enhance no records message logic for LG devices in download history
</commit_message>
<xml_diff>
--- a/documents/Calculo de Consumo por CDN.xlsx
+++ b/documents/Calculo de Consumo por CDN.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\Laravel\SCOTT\documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EED04426-EC60-415A-BD1D-06DB6384C05E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCD20196-7DE0-4C81-B913-406444A7F3C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -180,7 +180,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="8">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -279,11 +279,37 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -306,10 +332,29 @@
     <xf numFmtId="166" fontId="4" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="166" fontId="4" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="1" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="1" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="4" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -319,29 +364,16 @@
     <xf numFmtId="164" fontId="4" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="4" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="1" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="4" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="4" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="1" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="4" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="4" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="2" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="4" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="4" fillId="2" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -586,10 +618,10 @@
         <v>3</v>
       </c>
       <c r="B2" s="5">
-        <v>5051</v>
+        <v>5001</v>
       </c>
       <c r="C2" s="5">
-        <v>8023</v>
+        <v>7877</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="13.2">
@@ -609,109 +641,109 @@
       </c>
       <c r="B4" s="8">
         <f t="shared" ref="B4:C4" si="0">B2*B3</f>
-        <v>15153</v>
+        <v>15003</v>
       </c>
       <c r="C4" s="8">
         <f t="shared" si="0"/>
-        <v>16046</v>
+        <v>15754</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="13.2">
       <c r="A5" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="12">
+      <c r="B5" s="20">
         <f>B2+C2</f>
-        <v>13074</v>
-      </c>
-      <c r="C5" s="13"/>
+        <v>12878</v>
+      </c>
+      <c r="C5" s="14"/>
     </row>
     <row r="6" spans="1:3" ht="13.2">
       <c r="A6" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="12">
+      <c r="B6" s="20">
         <f>B4+C4</f>
-        <v>31199</v>
-      </c>
-      <c r="C6" s="13"/>
+        <v>30757</v>
+      </c>
+      <c r="C6" s="14"/>
     </row>
     <row r="7" spans="1:3" ht="13.2">
       <c r="A7" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="14">
+      <c r="B7" s="21">
         <v>3</v>
       </c>
-      <c r="C7" s="13"/>
+      <c r="C7" s="14"/>
     </row>
     <row r="8" spans="1:3" ht="13.2">
       <c r="A8" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="15">
+      <c r="B8" s="22">
         <f>B7*60*60/8/1024</f>
         <v>1.318359375</v>
       </c>
-      <c r="C8" s="13"/>
+      <c r="C8" s="14"/>
     </row>
     <row r="9" spans="1:3" ht="13.2">
       <c r="A9" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="16">
+      <c r="B9" s="23">
         <f>(B11/B6)*(1024)</f>
-        <v>35.241886848168157</v>
-      </c>
-      <c r="C9" s="13"/>
+        <v>35.748337867022087</v>
+      </c>
+      <c r="C9" s="14"/>
     </row>
     <row r="10" spans="1:3" ht="13.2">
       <c r="A10" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B10" s="23">
+      <c r="B10" s="15">
         <v>1000000</v>
       </c>
-      <c r="C10" s="13"/>
+      <c r="C10" s="14"/>
     </row>
     <row r="11" spans="1:3" ht="13.2">
       <c r="A11" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B11" s="19">
+      <c r="B11" s="16">
         <f>B10/931.32257461548</f>
         <v>1073.7418239999984</v>
       </c>
-      <c r="C11" s="13"/>
+      <c r="C11" s="14"/>
     </row>
     <row r="12" spans="1:3" ht="13.2">
       <c r="A12" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B12" s="18">
+      <c r="B12" s="13">
         <v>75000</v>
       </c>
-      <c r="C12" s="13"/>
+      <c r="C12" s="14"/>
     </row>
     <row r="13" spans="1:3" ht="13.2">
       <c r="A13" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B13" s="20">
+      <c r="B13" s="17">
         <f>B12/B11</f>
         <v>69.849193096161002</v>
       </c>
-      <c r="C13" s="13"/>
+      <c r="C13" s="14"/>
     </row>
     <row r="14" spans="1:3" ht="13.2">
       <c r="A14" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="B14" s="21">
+      <c r="B14" s="18">
         <f>B12/B6</f>
-        <v>2.4039232026667521</v>
-      </c>
-      <c r="C14" s="22"/>
+        <v>2.4384692915433885</v>
+      </c>
+      <c r="C14" s="19"/>
     </row>
     <row r="15" spans="1:3" ht="13.2">
       <c r="A15" s="10" t="s">
@@ -719,31 +751,31 @@
       </c>
       <c r="B15" s="11">
         <f>B14*B3</f>
-        <v>7.2117696080002567</v>
+        <v>7.3154078746301661</v>
       </c>
       <c r="C15" s="11">
         <f>B14*C3</f>
-        <v>4.8078464053335042</v>
+        <v>4.8769385830867771</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="15.75" customHeight="1">
       <c r="A16" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="B16" s="17">
+      <c r="B16" s="12">
         <f>B12/B5</f>
-        <v>5.736576411197797</v>
-      </c>
-      <c r="C16" s="17"/>
+        <v>5.8238856965367294</v>
+      </c>
+      <c r="C16" s="12"/>
     </row>
     <row r="17" spans="1:3" ht="15.75" customHeight="1">
       <c r="A17" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="B17" s="25">
+      <c r="B17" s="26">
         <v>390076.98</v>
       </c>
-      <c r="C17" s="25"/>
+      <c r="C17" s="27"/>
     </row>
     <row r="18" spans="1:3" ht="15.75" customHeight="1">
       <c r="A18" s="10" t="s">
@@ -751,9 +783,9 @@
       </c>
       <c r="B18" s="24">
         <f>B17/B6</f>
-        <v>12.502868040642328</v>
-      </c>
-      <c r="C18" s="24"/>
+        <v>12.68254316090646</v>
+      </c>
+      <c r="C18" s="25"/>
     </row>
     <row r="19" spans="1:3" ht="15.75" customHeight="1">
       <c r="A19" s="10" t="s">
@@ -761,17 +793,12 @@
       </c>
       <c r="B19" s="24">
         <f>B17/B5</f>
-        <v>29.836085360256998</v>
-      </c>
-      <c r="C19" s="24"/>
+        <v>30.290183258269916</v>
+      </c>
+      <c r="C19" s="25"/>
     </row>
   </sheetData>
   <mergeCells count="14">
-    <mergeCell ref="B17:C17"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="B12:C12"/>
     <mergeCell ref="B10:C10"/>
     <mergeCell ref="B11:C11"/>
     <mergeCell ref="B13:C13"/>
@@ -781,6 +808,11 @@
     <mergeCell ref="B7:C7"/>
     <mergeCell ref="B8:C8"/>
     <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="B12:C12"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>